<commit_message>
Use fake card digits (1234, 5678) in demo data
Replaces real card numbers with fictional ones so no confidential
account data is exposed in the public GitHub Pages demo.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_01_2026.xlsx
+++ b/demo_01_2026.xlsx
@@ -486,7 +486,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -520,7 +520,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -554,7 +554,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
@@ -588,7 +588,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -622,7 +622,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -656,7 +656,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
@@ -690,7 +690,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -724,7 +724,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
@@ -758,7 +758,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
@@ -792,7 +792,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
@@ -826,7 +826,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
@@ -860,7 +860,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
@@ -894,7 +894,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
@@ -928,7 +928,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
@@ -962,7 +962,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B20" s="1" t="n">
@@ -996,7 +996,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
@@ -1030,7 +1030,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B22" s="1" t="n">
@@ -1064,7 +1064,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B23" s="1" t="n">
@@ -1098,7 +1098,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B24" s="1" t="n">
@@ -1132,7 +1132,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B25" s="1" t="n">
@@ -1166,7 +1166,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B26" s="1" t="n">
@@ -1200,7 +1200,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B27" s="1" t="n">
@@ -1234,7 +1234,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B28" s="1" t="n">
@@ -1268,7 +1268,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B29" s="1" t="n">
@@ -1302,7 +1302,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B30" s="1" t="n">
@@ -1336,7 +1336,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B31" s="1" t="n">
@@ -1370,7 +1370,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B32" s="1" t="n">
@@ -1404,7 +1404,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B33" s="1" t="n">
@@ -1505,7 +1505,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B38" s="1" t="n">
@@ -1544,7 +1544,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8689</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="B39" s="1" t="n">
@@ -1583,7 +1583,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6138</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="B40" s="1" t="n">

</xml_diff>